<commit_message>
feat(gap-matrix): add O-RAN architecture standard analysis (R005-v16.00) to research gap matrix
</commit_message>
<xml_diff>
--- a/notes/gap_matrix/Gap Matrix.xlsx
+++ b/notes/gap_matrix/Gap Matrix.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Lessons ✒📝\Master\Term 3\Master's Theses\Paper\Paper_Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE496CB5-4C30-4271-A8B2-7B72B67E3B87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6BE8ACEB-259F-4BBE-AEE5-AE75920302D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="345" yWindow="3975" windowWidth="17475" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Gap Matrix" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <t>ID</t>
   </si>
@@ -60,25 +60,49 @@
     <t>Hamilton et al. (2017), "Inductive Representation Learning on Large Graphs," NIPS.</t>
   </si>
   <si>
-    <t>عدم توانایی مدل‌های سنتی در تولید امبدینگ برای گره‌های جدید (دیده‌نشده) بدون آموزش مجدد کل شبکه [۱، ۳، ۹].</t>
-  </si>
-  <si>
-    <t>GraphSAGE: یادگیری توابع تجمیع‌کننده (Aggregators) به جای یادگیری بردارهای ثابت برای هر گره [۱، ۶، ۱۳].</t>
-  </si>
-  <si>
-    <t>گراف‌های عظیم و پویا با ویژگی‌های غنی (مانند شبکه‌های استنادی، Reddit و تعاملات پروتئینی) [۳، ۲۸، ۳۲].</t>
-  </si>
-  <si>
-    <t>همسایگی محلی حاوی اطلاعات کافی برای تشخیص نقش گره است؛ استفاده از نمونه‌برداری یکنواخت برای ثابت نگه داشتن بار محاسباتی [۱، ۵، ۱۷، ۱۸].</t>
-  </si>
-  <si>
-    <t>نمره Micro-F1؛ مقایسه با DeepWalk و GCN؛ آزمایش بر روی گراف‌های کاملاً جدید (unseen graphs) [۸، ۲۴، ۲۷].</t>
-  </si>
-  <si>
-    <t>نمونه‌برداری تصادفی ممکن است همسایگان مهم را نادیده بگیرد؛ نیاز به ابعاد بالا برای شناسایی الگوهای ساختاری در بدترین حالت [۱۷، ۳۹، ۷۰].</t>
-  </si>
-  <si>
-    <t>امکان درک وضعیت سایت‌های جدید یا تغییرات توپولوژی در لایه rApp/xApp بدون وقفه در آموزش مدل [منبع ۹، منبع ۱۵].</t>
+    <t>پیاده‌سازی لایه‌های xApp و rApp در این چارچوب برای بهینه‌سازی ترافیک با استفاده از الگوریتم DRL+GNN و قابلیت Action Masking.</t>
+  </si>
+  <si>
+    <t>عدم پشتیبانی از مجازی‌سازی واحد رادیویی (O-RU) در این نسخه و پیچیدگی‌های محاسباتی ناشی از اجرای سیاست‌ها در بازه‌های زمانی میلی‌ثانیه‌ای.</t>
+  </si>
+  <si>
+    <t>شاخص‌های FCAPS (خطا، پیکربندی، حسابداری، عملکرد، امنیت) و تضمین توافق‌نامه سطح سرویس (SLA).</t>
+  </si>
+  <si>
+    <t>انطباق با استانداردهای 3GPP، استفاده از موجودیت‌های منطقی به‌جای فیزیکی و توانایی هدایت (Steering) در واسط A1.</t>
+  </si>
+  <si>
+    <t>معماری RAN با تمرکز بر مدیریت حلقه‌های کنترلی زمانی (Near-RT و Non-RT) و استفاده از سخت‌افزارهای تجاری آماده (COTS).</t>
+  </si>
+  <si>
+    <t>معماری تفکیک‌شده (Disaggregated) با واسط‌های باز (Open Interfaces) و کنترل‌کننده‌های هوشمند رادیویی (RIC).</t>
+  </si>
+  <si>
+    <t>انحصار سخت‌افزارهای بسته (Proprietary)، عدم تعامل‌پذیری بین سازندگان و فقدان هوشمندی داده‌محور در شبکه دسترسی رادیویی (RAN).</t>
+  </si>
+  <si>
+    <t>O-RAN.WG1.TS.OAD-R005-v16.00 (2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">عدم توانایی مدل‌های سنتی در تولید امبدینگ برای گره‌های جدید (دیده‌نشده) بدون آموزش مجدد کل شبکه </t>
+  </si>
+  <si>
+    <t>GraphSAGE: یادگیری توابع تجمیع‌کننده (Aggregators) به جای یادگیری بردارهای ثابت برای هر گره</t>
+  </si>
+  <si>
+    <t>گراف‌های عظیم و پویا با ویژگی‌های غنی (مانند شبکه‌های استنادی، Reddit و تعاملات پروتئینی)</t>
+  </si>
+  <si>
+    <t>همسایگی محلی حاوی اطلاعات کافی برای تشخیص نقش گره است؛ استفاده از نمونه‌برداری یکنواخت برای ثابت نگه داشتن بار محاسباتی</t>
+  </si>
+  <si>
+    <t>نمره Micro-F1؛ مقایسه با DeepWalk و GCN؛ آزمایش بر روی گراف‌های کاملاً جدید (unseen graphs)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">نمونه‌برداری تصادفی ممکن است همسایگان مهم را نادیده بگیرد؛ نیاز به ابعاد بالا برای شناسایی الگوهای ساختاری در بدترین حالت </t>
+  </si>
+  <si>
+    <t xml:space="preserve">امکان درک وضعیت سایت‌های جدید یا تغییرات توپولوژی در لایه rApp/xApp بدون وقفه در آموزش مدل </t>
   </si>
 </sst>
 </file>
@@ -86,7 +110,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="168" formatCode="[$-3000401]0"/>
+    <numFmt numFmtId="164" formatCode="[$-3000401]0"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -138,7 +162,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -163,154 +187,154 @@
     </dxf>
     <dxf>
       <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
         <b/>
         <i val="0"/>
         <strike val="0"/>
         <condense val="0"/>
         <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
         <u val="none"/>
@@ -337,18 +361,18 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{589AE12C-07C1-4442-8683-E464F1DA0A07}" name="Table1" displayName="Table1" ref="A1:I1048576" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{589AE12C-07C1-4442-8683-E464F1DA0A07}" name="Table1" displayName="Table1" ref="A1:I1048576" totalsRowShown="0" headerRowDxfId="10" dataDxfId="0">
   <autoFilter ref="A1:I1048576" xr:uid="{589AE12C-07C1-4442-8683-E464F1DA0A07}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{C8428E61-1742-4665-A3F8-195879308DDA}" name="ID" dataDxfId="10"/>
-    <tableColumn id="2" xr3:uid="{024D2EA6-98A5-41BB-883E-D54587041A90}" name="Reference" dataDxfId="9"/>
-    <tableColumn id="3" xr3:uid="{8F6729D5-0B92-463F-809C-FA0FB97FF064}" name="Core Problem" dataDxfId="8"/>
-    <tableColumn id="4" xr3:uid="{982CC9F5-640D-456A-B4F3-83A67A32F6BB}" name="Core Method" dataDxfId="7"/>
-    <tableColumn id="5" xr3:uid="{BEEB5F02-65A1-494D-A588-3482A53B9838}" name="Network Context" dataDxfId="6"/>
-    <tableColumn id="6" xr3:uid="{3500C5BC-26BA-43A1-A3F1-B48014112E9B}" name="Key Assumptions" dataDxfId="5"/>
-    <tableColumn id="9" xr3:uid="{B4ACD3B3-F80C-417B-A4DD-67A34578C796}" name="Metrics &amp; Evaluation" dataDxfId="4"/>
-    <tableColumn id="8" xr3:uid="{C50120FB-36C1-44C4-A383-2BF1C3BAE088}" name="Critical Limitation / Gap" dataDxfId="3"/>
-    <tableColumn id="7" xr3:uid="{912D7042-98B7-4696-BC68-3F2A2EF75F2C}" name="NeuroBottleneck Mapping" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{C8428E61-1742-4665-A3F8-195879308DDA}" name="ID" dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{024D2EA6-98A5-41BB-883E-D54587041A90}" name="Reference" dataDxfId="8"/>
+    <tableColumn id="3" xr3:uid="{8F6729D5-0B92-463F-809C-FA0FB97FF064}" name="Core Problem" dataDxfId="7"/>
+    <tableColumn id="4" xr3:uid="{982CC9F5-640D-456A-B4F3-83A67A32F6BB}" name="Core Method" dataDxfId="6"/>
+    <tableColumn id="5" xr3:uid="{BEEB5F02-65A1-494D-A588-3482A53B9838}" name="Network Context" dataDxfId="5"/>
+    <tableColumn id="6" xr3:uid="{3500C5BC-26BA-43A1-A3F1-B48014112E9B}" name="Key Assumptions" dataDxfId="4"/>
+    <tableColumn id="9" xr3:uid="{B4ACD3B3-F80C-417B-A4DD-67A34578C796}" name="Metrics &amp; Evaluation" dataDxfId="3"/>
+    <tableColumn id="8" xr3:uid="{C50120FB-36C1-44C4-A383-2BF1C3BAE088}" name="Critical Limitation / Gap" dataDxfId="2"/>
+    <tableColumn id="7" xr3:uid="{912D7042-98B7-4696-BC68-3F2A2EF75F2C}" name="NeuroBottleneck Mapping" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -620,19 +644,19 @@
   <dimension ref="A1:I3"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="21.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7" style="1" customWidth="1"/>
+    <col min="2" max="2" width="21.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="30" style="1" customWidth="1"/>
+    <col min="5" max="5" width="28.140625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="34.28515625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="33.42578125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="34.42578125" style="1" customWidth="1"/>
+    <col min="9" max="9" width="44.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="10" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="56.25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -661,7 +685,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="225" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" ht="93.75" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -669,30 +693,54 @@
         <v>9</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" ht="112.5" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>2</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs(standards): add ETSI TS 128 100 analysis, update Gap Matrix and Vocabulary
</commit_message>
<xml_diff>
--- a/notes/gap_matrix/Gap Matrix.xlsx
+++ b/notes/gap_matrix/Gap Matrix.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Lessons ✒📝\Master\Term 3\Master's Theses\Paper\Paper_Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6BE8ACEB-259F-4BBE-AEE5-AE75920302D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74715258-69BB-4ED6-BAE6-3FDF4C11D5F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="405" yWindow="735" windowWidth="17475" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Gap Matrix" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="33">
   <si>
     <t>ID</t>
   </si>
@@ -103,6 +103,30 @@
   </si>
   <si>
     <t xml:space="preserve">امکان درک وضعیت سایت‌های جدید یا تغییرات توپولوژی در لایه rApp/xApp بدون وقفه در آموزش مدل </t>
+  </si>
+  <si>
+    <t>ETSI TS 128 100 V19.0.0 (2025-10), "Levels of autonomous network"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">پیچیدگی فزاینده مدیریت شبکه 5G و هزینه‌های عملیاتی بالا (OPEX) به دلیل مدیریت دستی در مواجهه با تنوع سرویس‌ها و تعداد بالای دستگاه‌ها </t>
+  </si>
+  <si>
+    <t xml:space="preserve">چارچوب ارزیابی سطوح خودگردانی (L0 تا L5) بر پایه ابعاد سه‌گانه: سناریوها، قلمرو مدیریت و جریان کاری (شامل آگاهی، تحلیل، تصمیم و اجرا) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">سیستم‌های مدیریت و ارکستراسیون 3GPP در لایه‌های NE/NF، دامنه‌ای و بین‌دامنه‌ای </t>
+  </si>
+  <si>
+    <t xml:space="preserve">گذار گام‌به‌گام (Stepwise progression) از عملیات دستی به خودگردانی کامل؛ تقسیم وظایف بین انسان و سیستم در سطوح میانی </t>
+  </si>
+  <si>
+    <t xml:space="preserve">توانمندی سیستم در انجام خودکار وظایف جریان کاری (Workflow Tasks) و میزان تحقق نیت (Intent Fulfilment) اپراتور </t>
+  </si>
+  <si>
+    <t xml:space="preserve">عدم پوشش بخش «برنامه‌ریزی» (Planning) و لایه «سرویس ارتباطی»؛ تکیه بر نیت‌های تعریف شده توسط انسان تا سطح ۴ </t>
+  </si>
+  <si>
+    <t xml:space="preserve">انطباق معماری GNN+DRL با چرخه هوشمند استاندارد؛ استفاده از GNN برای آگاهی (Task D) و DRL برای تصمیم (Task I) جهت دستیابی به سطح ۴ خودگردانی </t>
   </si>
 </sst>
 </file>
@@ -187,21 +211,6 @@
     </dxf>
     <dxf>
       <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
         <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
@@ -226,6 +235,21 @@
         <strike val="0"/>
         <condense val="0"/>
         <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
         <u val="none"/>
@@ -361,18 +385,18 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{589AE12C-07C1-4442-8683-E464F1DA0A07}" name="Table1" displayName="Table1" ref="A1:I1048576" totalsRowShown="0" headerRowDxfId="10" dataDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{589AE12C-07C1-4442-8683-E464F1DA0A07}" name="Table1" displayName="Table1" ref="A1:I1048576" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9">
   <autoFilter ref="A1:I1048576" xr:uid="{589AE12C-07C1-4442-8683-E464F1DA0A07}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{C8428E61-1742-4665-A3F8-195879308DDA}" name="ID" dataDxfId="9"/>
-    <tableColumn id="2" xr3:uid="{024D2EA6-98A5-41BB-883E-D54587041A90}" name="Reference" dataDxfId="8"/>
-    <tableColumn id="3" xr3:uid="{8F6729D5-0B92-463F-809C-FA0FB97FF064}" name="Core Problem" dataDxfId="7"/>
-    <tableColumn id="4" xr3:uid="{982CC9F5-640D-456A-B4F3-83A67A32F6BB}" name="Core Method" dataDxfId="6"/>
-    <tableColumn id="5" xr3:uid="{BEEB5F02-65A1-494D-A588-3482A53B9838}" name="Network Context" dataDxfId="5"/>
-    <tableColumn id="6" xr3:uid="{3500C5BC-26BA-43A1-A3F1-B48014112E9B}" name="Key Assumptions" dataDxfId="4"/>
-    <tableColumn id="9" xr3:uid="{B4ACD3B3-F80C-417B-A4DD-67A34578C796}" name="Metrics &amp; Evaluation" dataDxfId="3"/>
-    <tableColumn id="8" xr3:uid="{C50120FB-36C1-44C4-A383-2BF1C3BAE088}" name="Critical Limitation / Gap" dataDxfId="2"/>
-    <tableColumn id="7" xr3:uid="{912D7042-98B7-4696-BC68-3F2A2EF75F2C}" name="NeuroBottleneck Mapping" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{C8428E61-1742-4665-A3F8-195879308DDA}" name="ID" dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{024D2EA6-98A5-41BB-883E-D54587041A90}" name="Reference" dataDxfId="7"/>
+    <tableColumn id="3" xr3:uid="{8F6729D5-0B92-463F-809C-FA0FB97FF064}" name="Core Problem" dataDxfId="6"/>
+    <tableColumn id="4" xr3:uid="{982CC9F5-640D-456A-B4F3-83A67A32F6BB}" name="Core Method" dataDxfId="5"/>
+    <tableColumn id="5" xr3:uid="{BEEB5F02-65A1-494D-A588-3482A53B9838}" name="Network Context" dataDxfId="4"/>
+    <tableColumn id="6" xr3:uid="{3500C5BC-26BA-43A1-A3F1-B48014112E9B}" name="Key Assumptions" dataDxfId="3"/>
+    <tableColumn id="9" xr3:uid="{B4ACD3B3-F80C-417B-A4DD-67A34578C796}" name="Metrics &amp; Evaluation" dataDxfId="2"/>
+    <tableColumn id="8" xr3:uid="{C50120FB-36C1-44C4-A383-2BF1C3BAE088}" name="Critical Limitation / Gap" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{912D7042-98B7-4696-BC68-3F2A2EF75F2C}" name="NeuroBottleneck Mapping" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -641,11 +665,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7" style="1" customWidth="1"/>
-    <col min="2" max="2" width="21.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.7109375" style="1" customWidth="1"/>
     <col min="3" max="3" width="26.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="30" style="1" customWidth="1"/>
     <col min="5" max="5" width="28.140625" style="1" customWidth="1"/>
@@ -743,6 +767,35 @@
         <v>10</v>
       </c>
     </row>
+    <row r="4" spans="1:9" ht="112.5" x14ac:dyDescent="0.25">
+      <c r="A4" s="1">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>

</xml_diff>

<commit_message>
docs: update AI-Core matrix with deep insights from GraphSAGE (NIPS 2017)
</commit_message>
<xml_diff>
--- a/notes/gap_matrix/Gap Matrix.xlsx
+++ b/notes/gap_matrix/Gap Matrix.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Lessons ✒📝\Master\Term 3\Master's Theses\Paper\Paper_Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74715258-69BB-4ED6-BAE6-3FDF4C11D5F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AE09D3A-81D2-4BE2-A5EF-D0EA7480D46E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="405" yWindow="735" windowWidth="17475" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="750" yWindow="1080" windowWidth="17475" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Gap Matrix" sheetId="1" r:id="rId1"/>
@@ -84,27 +84,6 @@
     <t>O-RAN.WG1.TS.OAD-R005-v16.00 (2026)</t>
   </si>
   <si>
-    <t xml:space="preserve">عدم توانایی مدل‌های سنتی در تولید امبدینگ برای گره‌های جدید (دیده‌نشده) بدون آموزش مجدد کل شبکه </t>
-  </si>
-  <si>
-    <t>GraphSAGE: یادگیری توابع تجمیع‌کننده (Aggregators) به جای یادگیری بردارهای ثابت برای هر گره</t>
-  </si>
-  <si>
-    <t>گراف‌های عظیم و پویا با ویژگی‌های غنی (مانند شبکه‌های استنادی، Reddit و تعاملات پروتئینی)</t>
-  </si>
-  <si>
-    <t>همسایگی محلی حاوی اطلاعات کافی برای تشخیص نقش گره است؛ استفاده از نمونه‌برداری یکنواخت برای ثابت نگه داشتن بار محاسباتی</t>
-  </si>
-  <si>
-    <t>نمره Micro-F1؛ مقایسه با DeepWalk و GCN؛ آزمایش بر روی گراف‌های کاملاً جدید (unseen graphs)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">نمونه‌برداری تصادفی ممکن است همسایگان مهم را نادیده بگیرد؛ نیاز به ابعاد بالا برای شناسایی الگوهای ساختاری در بدترین حالت </t>
-  </si>
-  <si>
-    <t xml:space="preserve">امکان درک وضعیت سایت‌های جدید یا تغییرات توپولوژی در لایه rApp/xApp بدون وقفه در آموزش مدل </t>
-  </si>
-  <si>
     <t>ETSI TS 128 100 V19.0.0 (2025-10), "Levels of autonomous network"</t>
   </si>
   <si>
@@ -127,6 +106,27 @@
   </si>
   <si>
     <t xml:space="preserve">انطباق معماری GNN+DRL با چرخه هوشمند استاندارد؛ استفاده از GNN برای آگاهی (Task D) و DRL برای تصمیم (Task I) جهت دستیابی به سطح ۴ خودگردانی </t>
+  </si>
+  <si>
+    <t xml:space="preserve">محدودیت روش‌های ترانسداکتیو در تعمیم‌پذیری به گره‌های دیده‌نشده و نیاز به آموزش مجدد کل گراف در شبکه‌های پویا </t>
+  </si>
+  <si>
+    <t xml:space="preserve">GraphSAGE: یادگیری توابع تجمیع‌کننده (بویژه Pooling) به جای بردارهای ایستا؛ استفاده از اتصال (Concatenation) برای حفظ هویت گره </t>
+  </si>
+  <si>
+    <t xml:space="preserve">گراف‌های عظیم و در حال تکامل (Evolving) با ویژگی‌های غنی (مانند تله‌متری و ظرفیت‌های لینک) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">همسایگی محلی حاوی نقش ساختاری است؛ ویژگی‌های گره (مانند خروجی گوموری-هو) فرآیند یادگیری را هدایت می‌کنند </t>
+  </si>
+  <si>
+    <t xml:space="preserve">نمره Micro-F1؛ پایداری در برابر نویز؛ سرعت استنتاج ۱۰۰ تا ۵۰۰ برابر بیشتر از DeepWalk (مناسب برای Near-RT) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">نمونه‌برداری تصادفی ممکن است یال‌های حساس ترافیکی را نادیده بگیرد؛ وابستگی شدید به کیفیت ویژگی‌های ورودی </t>
+  </si>
+  <si>
+    <t xml:space="preserve">لایه استخراج وضعیت (State) در xApp؛ تزریق دانش ریاضی به امبدینگ برای شناسایی بلادرنگ گلوگاه بدون نیاز به Retraining </t>
   </si>
 </sst>
 </file>
@@ -680,7 +680,7 @@
     <col min="10" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="37.5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -717,25 +717,25 @@
         <v>9</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="112.5" x14ac:dyDescent="0.25">
@@ -772,28 +772,28 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I4" s="1" t="s">
         <v>25</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="I4" s="1" t="s">
-        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: update AI-Core matrix with deep insights from PPO
</commit_message>
<xml_diff>
--- a/notes/gap_matrix/Gap Matrix.xlsx
+++ b/notes/gap_matrix/Gap Matrix.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Lessons ✒📝\Master\Term 3\Master's Theses\Paper\Paper_Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AE09D3A-81D2-4BE2-A5EF-D0EA7480D46E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EB76488-EC65-437F-A46B-0AA0E165DDC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="750" yWindow="1080" windowWidth="17475" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1095" yWindow="1425" windowWidth="17475" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Gap Matrix" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="41">
   <si>
     <t>ID</t>
   </si>
@@ -127,6 +127,51 @@
   </si>
   <si>
     <t xml:space="preserve">لایه استخراج وضعیت (State) در xApp؛ تزریق دانش ریاضی به امبدینگ برای شناسایی بلادرنگ گلوگاه بدون نیاز به Retraining </t>
+  </si>
+  <si>
+    <t>Schulman et al. (2017)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">به‌روزرسانی‌های مخرب و ناپایداری در یادگیری </t>
+  </si>
+  <si>
+    <t xml:space="preserve">PPO: تابع هدف مقید شده (Clipping) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">کنترل پیوسته و محیط‌های واکنشی </t>
+  </si>
+  <si>
+    <t>Clipping باعث پایداری و همگرایی یکنواخت می‌شود</t>
+  </si>
+  <si>
+    <t xml:space="preserve">میانگین پاداش؛ کارایی نمونه‌برداری </t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">حساسیت به هایپرپارامتر </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>اپسیلون</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> در محیط‌های پرنویز </t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">سیاست تصمیم‌گیری پایدار و ایمن در xApp </t>
   </si>
 </sst>
 </file>
@@ -665,7 +710,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7" style="1" customWidth="1"/>
@@ -796,6 +841,35 @@
         <v>25</v>
       </c>
     </row>
+    <row r="5" spans="1:9" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A5" s="3">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>

</xml_diff>

<commit_message>
docs: update AI-Core matrix with deep insights from DRLmeetsGNN
</commit_message>
<xml_diff>
--- a/notes/gap_matrix/Gap Matrix.xlsx
+++ b/notes/gap_matrix/Gap Matrix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Lessons ✒📝\Master\Term 3\Master's Theses\Paper\Paper_Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EB76488-EC65-437F-A46B-0AA0E165DDC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7793E5C-0C39-4D81-B952-743DBDC31166}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1095" yWindow="1425" windowWidth="17475" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="54">
   <si>
     <t>ID</t>
   </si>
@@ -60,45 +60,12 @@
     <t>Hamilton et al. (2017), "Inductive Representation Learning on Large Graphs," NIPS.</t>
   </si>
   <si>
-    <t>پیاده‌سازی لایه‌های xApp و rApp در این چارچوب برای بهینه‌سازی ترافیک با استفاده از الگوریتم DRL+GNN و قابلیت Action Masking.</t>
-  </si>
-  <si>
-    <t>عدم پشتیبانی از مجازی‌سازی واحد رادیویی (O-RU) در این نسخه و پیچیدگی‌های محاسباتی ناشی از اجرای سیاست‌ها در بازه‌های زمانی میلی‌ثانیه‌ای.</t>
-  </si>
-  <si>
-    <t>شاخص‌های FCAPS (خطا، پیکربندی، حسابداری، عملکرد، امنیت) و تضمین توافق‌نامه سطح سرویس (SLA).</t>
-  </si>
-  <si>
-    <t>انطباق با استانداردهای 3GPP، استفاده از موجودیت‌های منطقی به‌جای فیزیکی و توانایی هدایت (Steering) در واسط A1.</t>
-  </si>
-  <si>
-    <t>معماری RAN با تمرکز بر مدیریت حلقه‌های کنترلی زمانی (Near-RT و Non-RT) و استفاده از سخت‌افزارهای تجاری آماده (COTS).</t>
-  </si>
-  <si>
-    <t>معماری تفکیک‌شده (Disaggregated) با واسط‌های باز (Open Interfaces) و کنترل‌کننده‌های هوشمند رادیویی (RIC).</t>
-  </si>
-  <si>
-    <t>انحصار سخت‌افزارهای بسته (Proprietary)، عدم تعامل‌پذیری بین سازندگان و فقدان هوشمندی داده‌محور در شبکه دسترسی رادیویی (RAN).</t>
-  </si>
-  <si>
     <t>O-RAN.WG1.TS.OAD-R005-v16.00 (2026)</t>
   </si>
   <si>
     <t>ETSI TS 128 100 V19.0.0 (2025-10), "Levels of autonomous network"</t>
   </si>
   <si>
-    <t xml:space="preserve">پیچیدگی فزاینده مدیریت شبکه 5G و هزینه‌های عملیاتی بالا (OPEX) به دلیل مدیریت دستی در مواجهه با تنوع سرویس‌ها و تعداد بالای دستگاه‌ها </t>
-  </si>
-  <si>
-    <t xml:space="preserve">چارچوب ارزیابی سطوح خودگردانی (L0 تا L5) بر پایه ابعاد سه‌گانه: سناریوها، قلمرو مدیریت و جریان کاری (شامل آگاهی، تحلیل، تصمیم و اجرا) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">سیستم‌های مدیریت و ارکستراسیون 3GPP در لایه‌های NE/NF، دامنه‌ای و بین‌دامنه‌ای </t>
-  </si>
-  <si>
-    <t xml:space="preserve">گذار گام‌به‌گام (Stepwise progression) از عملیات دستی به خودگردانی کامل؛ تقسیم وظایف بین انسان و سیستم در سطوح میانی </t>
-  </si>
-  <si>
     <t xml:space="preserve">توانمندی سیستم در انجام خودکار وظایف جریان کاری (Workflow Tasks) و میزان تحقق نیت (Intent Fulfilment) اپراتور </t>
   </si>
   <si>
@@ -108,31 +75,10 @@
     <t xml:space="preserve">انطباق معماری GNN+DRL با چرخه هوشمند استاندارد؛ استفاده از GNN برای آگاهی (Task D) و DRL برای تصمیم (Task I) جهت دستیابی به سطح ۴ خودگردانی </t>
   </si>
   <si>
-    <t xml:space="preserve">محدودیت روش‌های ترانسداکتیو در تعمیم‌پذیری به گره‌های دیده‌نشده و نیاز به آموزش مجدد کل گراف در شبکه‌های پویا </t>
-  </si>
-  <si>
-    <t xml:space="preserve">GraphSAGE: یادگیری توابع تجمیع‌کننده (بویژه Pooling) به جای بردارهای ایستا؛ استفاده از اتصال (Concatenation) برای حفظ هویت گره </t>
-  </si>
-  <si>
-    <t xml:space="preserve">گراف‌های عظیم و در حال تکامل (Evolving) با ویژگی‌های غنی (مانند تله‌متری و ظرفیت‌های لینک) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">همسایگی محلی حاوی نقش ساختاری است؛ ویژگی‌های گره (مانند خروجی گوموری-هو) فرآیند یادگیری را هدایت می‌کنند </t>
-  </si>
-  <si>
     <t xml:space="preserve">نمره Micro-F1؛ پایداری در برابر نویز؛ سرعت استنتاج ۱۰۰ تا ۵۰۰ برابر بیشتر از DeepWalk (مناسب برای Near-RT) </t>
   </si>
   <si>
-    <t xml:space="preserve">نمونه‌برداری تصادفی ممکن است یال‌های حساس ترافیکی را نادیده بگیرد؛ وابستگی شدید به کیفیت ویژگی‌های ورودی </t>
-  </si>
-  <si>
-    <t xml:space="preserve">لایه استخراج وضعیت (State) در xApp؛ تزریق دانش ریاضی به امبدینگ برای شناسایی بلادرنگ گلوگاه بدون نیاز به Retraining </t>
-  </si>
-  <si>
     <t>Schulman et al. (2017)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">به‌روزرسانی‌های مخرب و ناپایداری در یادگیری </t>
   </si>
   <si>
     <t xml:space="preserve">PPO: تابع هدف مقید شده (Clipping) </t>
@@ -172,6 +118,120 @@
   </si>
   <si>
     <t xml:space="preserve">سیاست تصمیم‌گیری پایدار و ایمن در xApp </t>
+  </si>
+  <si>
+    <t>Almasan et al. (2022), "Deep reinforcement learning meets Graph Neural Networks," Computer Communications</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ناتوانی مدل‌ های DRL مبتنی بر شبکه ‌های عصبی سنتی (MLP/CNN) در تعمیم ‌پذیری به توپولوژی‌های جدید و دیده ‌نشده در زمان آموزش </t>
+  </si>
+  <si>
+    <t xml:space="preserve">به ‌روزرسانی‌ های مخرب و ناپایداری در یادگیری </t>
+  </si>
+  <si>
+    <t xml:space="preserve">پیچیدگی فزاینده مدیریت شبکه 5G و هزینه ‌های عملیاتی بالا (OPEX) به دلیل مدیریت دستی در مواجهه با تنوع سرویس‌ ها و تعداد بالای دستگاه ‌ها </t>
+  </si>
+  <si>
+    <t>تلفیق مستقیم GNN (معماری MPNN) در بدنه عامل DRL؛ طراحی فضای کنش ناوردا نسبت به جایگشت (Permutation Invariant) بر پایه مسیرهای کاندید</t>
+  </si>
+  <si>
+    <t>شبکه‌ های انتقال نوری (OTN) و زیرساخت ‌های مبتنی بر SDN با گراف‌ های مقیاس‌ بزرگ (تا ۱۰۰ گره)</t>
+  </si>
+  <si>
+    <t>شبکه ماهیت گرافی دارد؛ ویژگی‌ های سطح لینک (ظرفیت و بینابینی) برای درک وضعیت ترافیکی و اتخاذ تصمیم مسیریابی بهینه کافی هستند</t>
+  </si>
+  <si>
+    <t>مجموع پهنای باند تخصیص‌ یافته (Score)؛ مقایسه با مدل تئوریک Fluid؛ زمان استنتاج (Inference Time) در مقیاس میلی ‌ثانیه</t>
+  </si>
+  <si>
+    <t>افت عملکرد در مواجهه با داده‌ های خارج از توزیع (Out-of-distribution)؛ پیچیدگی در عیب ‌یابی به دلیل ماهیت جعبه ‌سیاه مدل عمیق</t>
+  </si>
+  <si>
+    <t xml:space="preserve">تأمین زیرساخت تعمیم ‌پذیری xApp در Near-RT RIC؛ تضمین تاب ‌آوری سیستم در سناریوی قطعی لینک (Fiber Cut) و تغییرات ناگهانی توپولوژی همراه اول </t>
+  </si>
+  <si>
+    <t xml:space="preserve">محدودیت روش‌های ترانسداکتیو در تعمیم‌ پذیری به گره ‌های دیده‌ نشده و نیاز به آموزش مجدد کل گراف در شبکه ‌های پویا </t>
+  </si>
+  <si>
+    <t xml:space="preserve">GraphSAGE: یادگیری توابع تجمیع ‌کننده (بویژه Pooling) به جای بردارهای ایستا؛ استفاده از اتصال (Concatenation) برای حفظ هویت گره </t>
+  </si>
+  <si>
+    <t xml:space="preserve">گراف ‌های عظیم و در حال تکامل (Evolving) با ویژگی‌ های غنی (مانند تله‌ متری و ظرفیت‌ های لینک) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">همسایگی محلی حاوی نقش ساختاری است؛ ویژگی ‌های گره (مانند خروجی گوموری-هو) فرآیند یادگیری را هدایت می‌کنند </t>
+  </si>
+  <si>
+    <t xml:space="preserve">نمونه ‌برداری تصادفی ممکن است یال‌ های حساس ترافیکی را نادیده بگیرد؛ وابستگی شدید به کیفیت ویژگی‌ های ورودی </t>
+  </si>
+  <si>
+    <t xml:space="preserve">لایه استخراج وضعیت (State) در xApp؛ تزریق دانش ریاضی به امبدینگ برای شناسایی بلادرنگ گلوگاه  بدون نیاز به Retraining </t>
+  </si>
+  <si>
+    <t>پیاده‌ سازی لایه‌های xApp و rApp در این چارچوب برای بهینه ‌سازی ترافیک با استفاده از الگوریتم DRL+GNN و قابلیت Action Masking.</t>
+  </si>
+  <si>
+    <t>عدم پشتیبانی از مجازی ‌سازی واحد رادیویی (O-RU) در این نسخه و پیچیدگی‌ های محاسباتی ناشی از اجرای سیاست ‌ها در بازه‌ های زمانی میلی ‌ثانیه‌ای.</t>
+  </si>
+  <si>
+    <t>شاخص ‌های FCAPS (خطا، پیکربندی، حسابداری، عملکرد، امنیت) و تضمین توافق ‌نامه سطح سرویس (SLA).</t>
+  </si>
+  <si>
+    <t>انطباق با استانداردهای 3GPP، استفاده از موجودیت‌ های منطقی به‌ جای فیزیکی و توانایی هدایت (Steering) در واسط A1.</t>
+  </si>
+  <si>
+    <t>معماری RAN با تمرکز بر مدیریت حلقه‌ های کنترلی زمانی (Near-RT و Non-RT) و استفاده از سخت ‌افزارهای تجاری آماده (COTS).</t>
+  </si>
+  <si>
+    <t>معماری تفکیک ‌شده (Disaggregated) با واسط ‌های باز (Open Interfaces) و کنترل ‌کننده‌ های هوشمند رادیویی (RIC).</t>
+  </si>
+  <si>
+    <t>انحصار سخت ‌افزارهای بسته (Proprietary)، عدم تعامل ‌پذیری بین سازندگان و فقدان هوشمندی داده‌ محور در شبکه دسترسی رادیویی (RAN).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">چارچوب ارزیابی سطوح خودگردانی (L0 تا L5) بر پایه ابعاد سه ‌گانه : سناریوها، قلمرو مدیریت و جریان کاری (شامل آگاهی، تحلیل، تصمیم و اجرا) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">سیستم‌ های مدیریت و ارکستراسیون 3GPP در لایه‌ های NE/NF، دامنه‌ ای و بین ‌دامنه‌ای </t>
+  </si>
+  <si>
+    <t xml:space="preserve">گذار گام ‌به‌ گام (Stepwise progression) از عملیات دستی به خودگردانی کامل؛ تقسیم وظایف بین انسان و سیستم در سطوح میانی </t>
+  </si>
+  <si>
+    <t xml:space="preserve">عدم پوشش بخش «برنامه‌ریزی» (Planning) و لایه «سرویس ارتباطی»؛ تکیه بر نیت ‌های تعریف شده توسط انسان تا سطح ۴ </t>
+  </si>
+  <si>
+    <t xml:space="preserve">سیاست تصمیم ‌گیری پایدار و ایمن در xApp </t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">حساسیت به هایپرپارامتر </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>اپسیلون</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> در محیط‌ های پرنویز </t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">میانگین پاداش؛ کارایی نمونه‌ برداری </t>
+  </si>
+  <si>
+    <t xml:space="preserve">کنترل پیوسته و محیط‌ های واکنشی </t>
   </si>
 </sst>
 </file>
@@ -223,7 +283,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -233,6 +293,12 @@
     </xf>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -710,7 +776,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I72"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7" style="1" customWidth="1"/>
@@ -761,26 +827,26 @@
       <c r="B2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>31</v>
+      <c r="C2" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>37</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="112.5" x14ac:dyDescent="0.25">
@@ -788,28 +854,28 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>40</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>10</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="112.5" x14ac:dyDescent="0.25">
@@ -817,58 +883,615 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C4" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A5" s="4">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="F5" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="D4" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="G4" s="1" t="s">
+      <c r="G5" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="112.5" x14ac:dyDescent="0.25">
+      <c r="A6" s="1">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="C6" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="I4" s="1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A5" s="3">
-        <v>4</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="I5" s="1" t="s">
-        <v>40</v>
-      </c>
+      <c r="D6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C7" s="5"/>
+      <c r="D7" s="5"/>
+      <c r="E7" s="5"/>
+      <c r="F7" s="5"/>
+      <c r="G7" s="5"/>
+      <c r="H7" s="5"/>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C8" s="5"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
+      <c r="F8" s="5"/>
+      <c r="G8" s="5"/>
+      <c r="H8" s="5"/>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C9" s="5"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
+      <c r="F9" s="5"/>
+      <c r="G9" s="5"/>
+      <c r="H9" s="5"/>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C10" s="5"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
+      <c r="F10" s="5"/>
+      <c r="G10" s="5"/>
+      <c r="H10" s="5"/>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C11" s="5"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
+      <c r="F11" s="5"/>
+      <c r="G11" s="5"/>
+      <c r="H11" s="5"/>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C12" s="5"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
+      <c r="F12" s="5"/>
+      <c r="G12" s="5"/>
+      <c r="H12" s="5"/>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C13" s="5"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
+      <c r="F13" s="5"/>
+      <c r="G13" s="5"/>
+      <c r="H13" s="5"/>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C14" s="5"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5"/>
+      <c r="F14" s="5"/>
+      <c r="G14" s="5"/>
+      <c r="H14" s="5"/>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C15" s="5"/>
+      <c r="D15" s="5"/>
+      <c r="E15" s="5"/>
+      <c r="F15" s="5"/>
+      <c r="G15" s="5"/>
+      <c r="H15" s="5"/>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C16" s="5"/>
+      <c r="D16" s="5"/>
+      <c r="E16" s="5"/>
+      <c r="F16" s="5"/>
+      <c r="G16" s="5"/>
+      <c r="H16" s="5"/>
+    </row>
+    <row r="17" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C17" s="5"/>
+      <c r="D17" s="5"/>
+      <c r="E17" s="5"/>
+      <c r="F17" s="5"/>
+      <c r="G17" s="5"/>
+      <c r="H17" s="5"/>
+    </row>
+    <row r="18" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C18" s="5"/>
+      <c r="D18" s="5"/>
+      <c r="E18" s="5"/>
+      <c r="F18" s="5"/>
+      <c r="G18" s="5"/>
+      <c r="H18" s="5"/>
+    </row>
+    <row r="19" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C19" s="5"/>
+      <c r="D19" s="5"/>
+      <c r="E19" s="5"/>
+      <c r="F19" s="5"/>
+      <c r="G19" s="5"/>
+      <c r="H19" s="5"/>
+    </row>
+    <row r="20" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C20" s="5"/>
+      <c r="D20" s="5"/>
+      <c r="E20" s="5"/>
+      <c r="F20" s="5"/>
+      <c r="G20" s="5"/>
+      <c r="H20" s="5"/>
+    </row>
+    <row r="21" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C21" s="5"/>
+      <c r="D21" s="5"/>
+      <c r="E21" s="5"/>
+      <c r="F21" s="5"/>
+      <c r="G21" s="5"/>
+      <c r="H21" s="5"/>
+    </row>
+    <row r="22" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C22" s="5"/>
+      <c r="D22" s="5"/>
+      <c r="E22" s="5"/>
+      <c r="F22" s="5"/>
+      <c r="G22" s="5"/>
+      <c r="H22" s="5"/>
+    </row>
+    <row r="23" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C23" s="5"/>
+      <c r="D23" s="5"/>
+      <c r="E23" s="5"/>
+      <c r="F23" s="5"/>
+      <c r="G23" s="5"/>
+      <c r="H23" s="5"/>
+    </row>
+    <row r="24" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C24" s="5"/>
+      <c r="D24" s="5"/>
+      <c r="E24" s="5"/>
+      <c r="F24" s="5"/>
+      <c r="G24" s="5"/>
+      <c r="H24" s="5"/>
+    </row>
+    <row r="25" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C25" s="5"/>
+      <c r="D25" s="5"/>
+      <c r="E25" s="5"/>
+      <c r="F25" s="5"/>
+      <c r="G25" s="5"/>
+      <c r="H25" s="5"/>
+    </row>
+    <row r="26" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C26" s="5"/>
+      <c r="D26" s="5"/>
+      <c r="E26" s="5"/>
+      <c r="F26" s="5"/>
+      <c r="G26" s="5"/>
+      <c r="H26" s="5"/>
+    </row>
+    <row r="27" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C27" s="5"/>
+      <c r="D27" s="5"/>
+      <c r="E27" s="5"/>
+      <c r="F27" s="5"/>
+      <c r="G27" s="5"/>
+      <c r="H27" s="5"/>
+    </row>
+    <row r="28" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C28" s="5"/>
+      <c r="D28" s="5"/>
+      <c r="E28" s="5"/>
+      <c r="F28" s="5"/>
+      <c r="G28" s="5"/>
+      <c r="H28" s="5"/>
+    </row>
+    <row r="29" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C29" s="5"/>
+      <c r="D29" s="5"/>
+      <c r="E29" s="5"/>
+      <c r="F29" s="5"/>
+      <c r="G29" s="5"/>
+      <c r="H29" s="5"/>
+    </row>
+    <row r="30" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C30" s="5"/>
+      <c r="D30" s="5"/>
+      <c r="E30" s="5"/>
+      <c r="F30" s="5"/>
+      <c r="G30" s="5"/>
+      <c r="H30" s="5"/>
+    </row>
+    <row r="31" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C31" s="5"/>
+      <c r="D31" s="5"/>
+      <c r="E31" s="5"/>
+      <c r="F31" s="5"/>
+      <c r="G31" s="5"/>
+      <c r="H31" s="5"/>
+    </row>
+    <row r="32" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C32" s="5"/>
+      <c r="D32" s="5"/>
+      <c r="E32" s="5"/>
+      <c r="F32" s="5"/>
+      <c r="G32" s="5"/>
+      <c r="H32" s="5"/>
+    </row>
+    <row r="33" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C33" s="5"/>
+      <c r="D33" s="5"/>
+      <c r="E33" s="5"/>
+      <c r="F33" s="5"/>
+      <c r="G33" s="5"/>
+      <c r="H33" s="5"/>
+    </row>
+    <row r="34" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C34" s="5"/>
+      <c r="D34" s="5"/>
+      <c r="E34" s="5"/>
+      <c r="F34" s="5"/>
+      <c r="G34" s="5"/>
+      <c r="H34" s="5"/>
+    </row>
+    <row r="35" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C35" s="5"/>
+      <c r="D35" s="5"/>
+      <c r="E35" s="5"/>
+      <c r="F35" s="5"/>
+      <c r="G35" s="5"/>
+      <c r="H35" s="5"/>
+    </row>
+    <row r="36" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C36" s="5"/>
+      <c r="D36" s="5"/>
+      <c r="E36" s="5"/>
+      <c r="F36" s="5"/>
+      <c r="G36" s="5"/>
+      <c r="H36" s="5"/>
+    </row>
+    <row r="37" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C37" s="5"/>
+      <c r="D37" s="5"/>
+      <c r="E37" s="5"/>
+      <c r="F37" s="5"/>
+      <c r="G37" s="5"/>
+      <c r="H37" s="5"/>
+    </row>
+    <row r="38" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C38" s="5"/>
+      <c r="D38" s="5"/>
+      <c r="E38" s="5"/>
+      <c r="F38" s="5"/>
+      <c r="G38" s="5"/>
+      <c r="H38" s="5"/>
+    </row>
+    <row r="39" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C39" s="5"/>
+      <c r="D39" s="5"/>
+      <c r="E39" s="5"/>
+      <c r="F39" s="5"/>
+      <c r="G39" s="5"/>
+      <c r="H39" s="5"/>
+    </row>
+    <row r="40" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C40" s="5"/>
+      <c r="D40" s="5"/>
+      <c r="E40" s="5"/>
+      <c r="F40" s="5"/>
+      <c r="G40" s="5"/>
+      <c r="H40" s="5"/>
+    </row>
+    <row r="41" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C41" s="5"/>
+      <c r="D41" s="5"/>
+      <c r="E41" s="5"/>
+      <c r="F41" s="5"/>
+      <c r="G41" s="5"/>
+      <c r="H41" s="5"/>
+    </row>
+    <row r="42" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C42" s="5"/>
+      <c r="D42" s="5"/>
+      <c r="E42" s="5"/>
+      <c r="F42" s="5"/>
+      <c r="G42" s="5"/>
+      <c r="H42" s="5"/>
+    </row>
+    <row r="43" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C43" s="5"/>
+      <c r="D43" s="5"/>
+      <c r="E43" s="5"/>
+      <c r="F43" s="5"/>
+      <c r="G43" s="5"/>
+      <c r="H43" s="5"/>
+    </row>
+    <row r="44" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C44" s="5"/>
+      <c r="D44" s="5"/>
+      <c r="E44" s="5"/>
+      <c r="F44" s="5"/>
+      <c r="G44" s="5"/>
+      <c r="H44" s="5"/>
+    </row>
+    <row r="45" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C45" s="5"/>
+      <c r="D45" s="5"/>
+      <c r="E45" s="5"/>
+      <c r="F45" s="5"/>
+      <c r="G45" s="5"/>
+      <c r="H45" s="5"/>
+    </row>
+    <row r="46" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C46" s="5"/>
+      <c r="D46" s="5"/>
+      <c r="E46" s="5"/>
+      <c r="F46" s="5"/>
+      <c r="G46" s="5"/>
+      <c r="H46" s="5"/>
+    </row>
+    <row r="47" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C47" s="5"/>
+      <c r="D47" s="5"/>
+      <c r="E47" s="5"/>
+      <c r="F47" s="5"/>
+      <c r="G47" s="5"/>
+      <c r="H47" s="5"/>
+    </row>
+    <row r="48" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C48" s="5"/>
+      <c r="D48" s="5"/>
+      <c r="E48" s="5"/>
+      <c r="F48" s="5"/>
+      <c r="G48" s="5"/>
+      <c r="H48" s="5"/>
+    </row>
+    <row r="49" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C49" s="5"/>
+      <c r="D49" s="5"/>
+      <c r="E49" s="5"/>
+      <c r="F49" s="5"/>
+      <c r="G49" s="5"/>
+      <c r="H49" s="5"/>
+    </row>
+    <row r="50" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C50" s="5"/>
+      <c r="D50" s="5"/>
+      <c r="E50" s="5"/>
+      <c r="F50" s="5"/>
+      <c r="G50" s="5"/>
+      <c r="H50" s="5"/>
+    </row>
+    <row r="51" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C51" s="5"/>
+      <c r="D51" s="5"/>
+      <c r="E51" s="5"/>
+      <c r="F51" s="5"/>
+      <c r="G51" s="5"/>
+      <c r="H51" s="5"/>
+    </row>
+    <row r="52" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C52" s="5"/>
+      <c r="D52" s="5"/>
+      <c r="E52" s="5"/>
+      <c r="F52" s="5"/>
+      <c r="G52" s="5"/>
+      <c r="H52" s="5"/>
+    </row>
+    <row r="53" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C53" s="5"/>
+      <c r="D53" s="5"/>
+      <c r="E53" s="5"/>
+      <c r="F53" s="5"/>
+      <c r="G53" s="5"/>
+      <c r="H53" s="5"/>
+    </row>
+    <row r="54" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C54" s="5"/>
+      <c r="D54" s="5"/>
+      <c r="E54" s="5"/>
+      <c r="F54" s="5"/>
+      <c r="G54" s="5"/>
+      <c r="H54" s="5"/>
+    </row>
+    <row r="55" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C55" s="5"/>
+      <c r="D55" s="5"/>
+      <c r="E55" s="5"/>
+      <c r="F55" s="5"/>
+      <c r="G55" s="5"/>
+      <c r="H55" s="5"/>
+    </row>
+    <row r="56" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C56" s="5"/>
+      <c r="D56" s="5"/>
+      <c r="E56" s="5"/>
+      <c r="F56" s="5"/>
+      <c r="G56" s="5"/>
+      <c r="H56" s="5"/>
+    </row>
+    <row r="57" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C57" s="5"/>
+      <c r="D57" s="5"/>
+      <c r="E57" s="5"/>
+      <c r="F57" s="5"/>
+      <c r="G57" s="5"/>
+      <c r="H57" s="5"/>
+    </row>
+    <row r="58" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C58" s="5"/>
+      <c r="D58" s="5"/>
+      <c r="E58" s="5"/>
+      <c r="F58" s="5"/>
+      <c r="G58" s="5"/>
+      <c r="H58" s="5"/>
+    </row>
+    <row r="59" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C59" s="5"/>
+      <c r="D59" s="5"/>
+      <c r="E59" s="5"/>
+      <c r="F59" s="5"/>
+      <c r="G59" s="5"/>
+      <c r="H59" s="5"/>
+    </row>
+    <row r="60" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C60" s="5"/>
+      <c r="D60" s="5"/>
+      <c r="E60" s="5"/>
+      <c r="F60" s="5"/>
+      <c r="G60" s="5"/>
+      <c r="H60" s="5"/>
+    </row>
+    <row r="61" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C61" s="5"/>
+      <c r="D61" s="5"/>
+      <c r="E61" s="5"/>
+      <c r="F61" s="5"/>
+      <c r="G61" s="5"/>
+      <c r="H61" s="5"/>
+    </row>
+    <row r="62" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C62" s="5"/>
+      <c r="D62" s="5"/>
+      <c r="E62" s="5"/>
+      <c r="F62" s="5"/>
+      <c r="G62" s="5"/>
+      <c r="H62" s="5"/>
+    </row>
+    <row r="63" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C63" s="5"/>
+      <c r="D63" s="5"/>
+      <c r="E63" s="5"/>
+      <c r="F63" s="5"/>
+      <c r="G63" s="5"/>
+      <c r="H63" s="5"/>
+    </row>
+    <row r="64" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C64" s="5"/>
+      <c r="D64" s="5"/>
+      <c r="E64" s="5"/>
+      <c r="F64" s="5"/>
+      <c r="G64" s="5"/>
+      <c r="H64" s="5"/>
+    </row>
+    <row r="65" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C65" s="5"/>
+      <c r="D65" s="5"/>
+      <c r="E65" s="5"/>
+      <c r="F65" s="5"/>
+      <c r="G65" s="5"/>
+      <c r="H65" s="5"/>
+    </row>
+    <row r="66" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C66" s="5"/>
+      <c r="D66" s="5"/>
+      <c r="E66" s="5"/>
+      <c r="F66" s="5"/>
+      <c r="G66" s="5"/>
+      <c r="H66" s="5"/>
+    </row>
+    <row r="67" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C67" s="5"/>
+      <c r="D67" s="5"/>
+      <c r="E67" s="5"/>
+      <c r="F67" s="5"/>
+      <c r="G67" s="5"/>
+      <c r="H67" s="5"/>
+    </row>
+    <row r="68" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C68" s="5"/>
+      <c r="D68" s="5"/>
+      <c r="E68" s="5"/>
+      <c r="F68" s="5"/>
+      <c r="G68" s="5"/>
+      <c r="H68" s="5"/>
+    </row>
+    <row r="69" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C69" s="5"/>
+      <c r="D69" s="5"/>
+      <c r="E69" s="5"/>
+      <c r="F69" s="5"/>
+      <c r="G69" s="5"/>
+      <c r="H69" s="5"/>
+    </row>
+    <row r="70" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C70" s="5"/>
+      <c r="D70" s="5"/>
+      <c r="E70" s="5"/>
+      <c r="F70" s="5"/>
+      <c r="G70" s="5"/>
+      <c r="H70" s="5"/>
+    </row>
+    <row r="71" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C71" s="5"/>
+      <c r="D71" s="5"/>
+      <c r="E71" s="5"/>
+      <c r="F71" s="5"/>
+      <c r="G71" s="5"/>
+      <c r="H71" s="5"/>
+    </row>
+    <row r="72" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C72" s="5"/>
+      <c r="D72" s="5"/>
+      <c r="E72" s="5"/>
+      <c r="F72" s="5"/>
+      <c r="G72" s="5"/>
+      <c r="H72" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>